<commit_message>
Add create and import functionality for Komoditas
Implemented manual and Excel import creation of Komoditas in the controller, updated the model to include 'edited_by', and enhanced the Vue page to support both creation modes and preview of import data. Also added the corresponding route and updated the Komoditas Excel template.
</commit_message>
<xml_diff>
--- a/public/document/Template Komoditas.xlsx
+++ b/public/document/Template Komoditas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\karlota-webbps\public\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D896DC1A-807B-46CB-A657-68327B274441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5129B526-4A82-4811-9344-54266693D08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DFF1197E-F150-4B02-B263-72EEA873BFD4}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>satuan</t>
   </si>
   <si>
-    <t>subsektor</t>
-  </si>
-  <si>
     <t>(jenis tipe bisa diliat di-sheet metadata)</t>
   </si>
   <si>
@@ -289,6 +286,9 @@
   </si>
   <si>
     <t>(bisa diisikan atau tidak)</t>
+  </si>
+  <si>
+    <t>subsector_id</t>
   </si>
 </sst>
 </file>
@@ -424,7 +424,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -437,8 +437,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -447,9 +449,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -808,20 +807,20 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -841,40 +840,38 @@
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9" t="s">
-        <v>9</v>
+      <c r="C3" s="8" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
+      <c r="C4" s="8"/>
     </row>
     <row r="5" spans="1:3" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="12"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -882,7 +879,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -890,7 +887,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -898,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -906,7 +903,7 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -914,7 +911,7 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -922,7 +919,7 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -930,7 +927,7 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -938,7 +935,7 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -946,7 +943,7 @@
         <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -954,7 +951,7 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -962,7 +959,7 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -970,7 +967,7 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -978,7 +975,7 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -986,7 +983,7 @@
         <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -994,7 +991,7 @@
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1002,7 +999,7 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -1010,7 +1007,7 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -1018,7 +1015,7 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -1026,7 +1023,7 @@
         <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -1034,7 +1031,7 @@
         <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -1042,7 +1039,7 @@
         <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -1050,7 +1047,7 @@
         <v>22</v>
       </c>
       <c r="B29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -1058,7 +1055,7 @@
         <v>23</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -1066,7 +1063,7 @@
         <v>24</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -1074,7 +1071,7 @@
         <v>25</v>
       </c>
       <c r="B32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -1082,7 +1079,7 @@
         <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -1090,7 +1087,7 @@
         <v>27</v>
       </c>
       <c r="B34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -1098,7 +1095,7 @@
         <v>28</v>
       </c>
       <c r="B35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -1106,7 +1103,7 @@
         <v>29</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -1114,7 +1111,7 @@
         <v>30</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -1122,7 +1119,7 @@
         <v>31</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -1130,7 +1127,7 @@
         <v>32</v>
       </c>
       <c r="B39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -1138,7 +1135,7 @@
         <v>33</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -1146,7 +1143,7 @@
         <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -1154,7 +1151,7 @@
         <v>35</v>
       </c>
       <c r="B42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -1162,7 +1159,7 @@
         <v>36</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -1170,7 +1167,7 @@
         <v>37</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -1178,7 +1175,7 @@
         <v>38</v>
       </c>
       <c r="B45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -1186,7 +1183,7 @@
         <v>39</v>
       </c>
       <c r="B46" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -1194,7 +1191,7 @@
         <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -1202,7 +1199,7 @@
         <v>41</v>
       </c>
       <c r="B48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -1210,7 +1207,7 @@
         <v>42</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -1218,7 +1215,7 @@
         <v>43</v>
       </c>
       <c r="B50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -1226,7 +1223,7 @@
         <v>44</v>
       </c>
       <c r="B51" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -1234,7 +1231,7 @@
         <v>45</v>
       </c>
       <c r="B52" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -1242,7 +1239,7 @@
         <v>46</v>
       </c>
       <c r="B53" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -1250,7 +1247,7 @@
         <v>47</v>
       </c>
       <c r="B54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -1258,7 +1255,7 @@
         <v>48</v>
       </c>
       <c r="B55" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -1266,7 +1263,7 @@
         <v>49</v>
       </c>
       <c r="B56" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -1274,7 +1271,7 @@
         <v>50</v>
       </c>
       <c r="B57" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -1282,7 +1279,7 @@
         <v>51</v>
       </c>
       <c r="B58" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -1290,7 +1287,7 @@
         <v>52</v>
       </c>
       <c r="B59" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -1298,7 +1295,7 @@
         <v>53</v>
       </c>
       <c r="B60" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -1306,7 +1303,7 @@
         <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -1314,7 +1311,7 @@
         <v>55</v>
       </c>
       <c r="B62" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -1322,7 +1319,7 @@
         <v>56</v>
       </c>
       <c r="B63" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -1330,7 +1327,7 @@
         <v>57</v>
       </c>
       <c r="B64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -1338,7 +1335,7 @@
         <v>58</v>
       </c>
       <c r="B65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -1346,7 +1343,7 @@
         <v>59</v>
       </c>
       <c r="B66" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -1354,7 +1351,7 @@
         <v>60</v>
       </c>
       <c r="B67" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -1362,7 +1359,7 @@
         <v>61</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -1370,7 +1367,7 @@
         <v>62</v>
       </c>
       <c r="B69" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -1378,7 +1375,7 @@
         <v>63</v>
       </c>
       <c r="B70" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -1386,7 +1383,7 @@
         <v>64</v>
       </c>
       <c r="B71" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -1394,7 +1391,7 @@
         <v>65</v>
       </c>
       <c r="B72" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -1402,7 +1399,7 @@
         <v>66</v>
       </c>
       <c r="B73" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -1410,7 +1407,7 @@
         <v>67</v>
       </c>
       <c r="B74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -1418,7 +1415,7 @@
         <v>68</v>
       </c>
       <c r="B75" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -1426,7 +1423,7 @@
         <v>69</v>
       </c>
       <c r="B76" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Harga Dasar management to Komoditas and IH
Introduces HargaDasar model and integrates harga dasar (base price) management into Komoditas and Indeks Harga workflows. Updates controllers to handle harga dasar data, modifies Komoditas and DasarIdx Vue pages to display and input harga dasar, and updates the Komoditas Excel template. This enables tracking and editing of base prices for commodities.
</commit_message>
<xml_diff>
--- a/public/document/Template Komoditas.xlsx
+++ b/public/document/Template Komoditas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\karlota-webbps\public\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5129B526-4A82-4811-9344-54266693D08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F2D05E-23D1-4267-8EE7-70B1BF5F2BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DFF1197E-F150-4B02-B263-72EEA873BFD4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DFF1197E-F150-4B02-B263-72EEA873BFD4}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>label</t>
   </si>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t>subsector_id</t>
+  </si>
+  <si>
+    <t>isian harga dasar dari komoditas (bisa diisi atau tidak)</t>
+  </si>
+  <si>
+    <t>harga_dasar (2010)</t>
   </si>
 </sst>
 </file>
@@ -784,16 +790,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{977FEE0D-4150-4255-ABC9-97FDCBA4333D}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
     <col min="2" max="2" width="23.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="37" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="53.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -809,8 +816,11 @@
       <c r="E1" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
         <v>82</v>
@@ -821,6 +831,9 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor harga_dasar to harga_konstan in Komoditas
Renamed all references of 'harga_dasar' to 'harga_konstan' in KomoditasController and Vue component for consistency. Updated migration to change the structure of 'master_harga' table, replacing the old column with a new decimal 'harga_konstan'. Adjusted Komoditas template and UI to reflect the new naming and display format.
</commit_message>
<xml_diff>
--- a/public/document/Template Komoditas.xlsx
+++ b/public/document/Template Komoditas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp\htdocs\karlota-webbps\public\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F2D05E-23D1-4267-8EE7-70B1BF5F2BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373363F7-9FA3-4F59-96B3-A1E4A0C1809E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DFF1197E-F150-4B02-B263-72EEA873BFD4}"/>
   </bookViews>
@@ -294,7 +294,7 @@
     <t>isian harga dasar dari komoditas (bisa diisi atau tidak)</t>
   </si>
   <si>
-    <t>harga_dasar (2010)</t>
+    <t>harga_konstan</t>
   </si>
 </sst>
 </file>

</xml_diff>